<commit_message>
Hp test cases and sprint 115 changes
</commit_message>
<xml_diff>
--- a/src/main/resources/excel_data/UserUpload.xlsx
+++ b/src/main/resources/excel_data/UserUpload.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vishmitha G\Documents\Automation\ctp-contiplus-web-qa-automation-java\src\main\resources\excel_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF5E76A-FC6D-4AEB-904A-33F378504FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACB7C9D-C87F-4419-B229-6ECE38BC7023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>Fullname</t>
   </si>
@@ -74,10 +74,7 @@
     <t>+919234567890</t>
   </si>
   <si>
-    <t>vtesttemp1</t>
-  </si>
-  <si>
-    <t>2customTemplate</t>
+    <t>uploadcustomTemplate</t>
   </si>
 </sst>
 </file>
@@ -163,9 +160,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -203,7 +200,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -309,7 +306,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -451,7 +448,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -516,7 +513,7 @@
         <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="31.2" x14ac:dyDescent="0.3">
@@ -533,7 +530,7 @@
         <v>13</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>